<commit_message>
debug commit for claude
</commit_message>
<xml_diff>
--- a/castle_level_1.xlsx
+++ b/castle_level_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\C++ Projects\castle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA52DD2-C08E-40C8-AB52-C142C7B1535E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F153FF-2054-4CF0-B044-CB76046518CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1005" yWindow="420" windowWidth="21600" windowHeight="13185" xr2:uid="{78F35DAF-77DF-4856-BA13-D4A6793299ED}"/>
+    <workbookView xWindow="28680" yWindow="1680" windowWidth="29040" windowHeight="15990" xr2:uid="{78F35DAF-77DF-4856-BA13-D4A6793299ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -106,7 +106,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -122,6 +122,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -157,8 +163,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,13 +518,13 @@
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H3" s="2"/>
@@ -532,7 +538,7 @@
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="G4" s="2"/>
@@ -545,22 +551,22 @@
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -570,16 +576,16 @@
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>5</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -587,24 +593,24 @@
       <c r="A7">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="1" t="s">
         <v>12</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -612,24 +618,24 @@
       <c r="A8">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -637,22 +643,22 @@
       <c r="A9">
         <v>6</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="1" t="s">
         <v>20</v>
       </c>
     </row>
@@ -663,7 +669,7 @@
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="2"/>

</xml_diff>